<commit_message>
Update candidate charts and all candidates list
</commit_message>
<xml_diff>
--- a/output/latest/all_candidates_latest.xlsx
+++ b/output/latest/all_candidates_latest.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="all_candidates" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="true_breakout" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="range_rebound" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="revenue_pullback" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="pullback_rebound" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="all_candidates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="true_breakout" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="range_rebound" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="revenue_pullback" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pullback_rebound" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update official warrant flow data
</commit_message>
<xml_diff>
--- a/output/latest/all_candidates_latest.xlsx
+++ b/output/latest/all_candidates_latest.xlsx
@@ -1068,7 +1068,7 @@
       </c>
       <c r="BN3" t="inlineStr"/>
       <c r="BO3" t="n">
-        <v>0</v>
+        <v>12822110</v>
       </c>
       <c r="BP3" t="n">
         <v>0</v>
@@ -1081,12 +1081,12 @@
       </c>
       <c r="BU3" t="inlineStr">
         <is>
-          <t>中信</t>
+          <t>富邦</t>
         </is>
       </c>
       <c r="BV3" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="BN7" t="inlineStr"/>
       <c r="BO7" t="n">
-        <v>0</v>
+        <v>3310770</v>
       </c>
       <c r="BP7" t="n">
         <v>0</v>
@@ -1659,10 +1659,14 @@
       <c r="BT7" t="n">
         <v>0</v>
       </c>
-      <c r="BU7" t="inlineStr"/>
+      <c r="BU7" t="inlineStr">
+        <is>
+          <t>群益</t>
+        </is>
+      </c>
       <c r="BV7" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1808,7 @@
       </c>
       <c r="BN8" t="inlineStr"/>
       <c r="BO8" t="n">
-        <v>0</v>
+        <v>5411230</v>
       </c>
       <c r="BP8" t="n">
         <v>0</v>
@@ -1815,10 +1819,14 @@
       <c r="BT8" t="n">
         <v>0</v>
       </c>
-      <c r="BU8" t="inlineStr"/>
+      <c r="BU8" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV8" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2108,7 @@
       </c>
       <c r="BN10" t="inlineStr"/>
       <c r="BO10" t="n">
-        <v>0</v>
+        <v>5112570</v>
       </c>
       <c r="BP10" t="n">
         <v>0</v>
@@ -2111,10 +2119,14 @@
       <c r="BT10" t="n">
         <v>0</v>
       </c>
-      <c r="BU10" t="inlineStr"/>
+      <c r="BU10" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV10" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -2396,7 +2408,7 @@
       </c>
       <c r="BN12" t="inlineStr"/>
       <c r="BO12" t="n">
-        <v>0</v>
+        <v>12839340</v>
       </c>
       <c r="BP12" t="n">
         <v>0</v>
@@ -2407,10 +2419,14 @@
       <c r="BT12" t="n">
         <v>0</v>
       </c>
-      <c r="BU12" t="inlineStr"/>
+      <c r="BU12" t="inlineStr">
+        <is>
+          <t>統一</t>
+        </is>
+      </c>
       <c r="BV12" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -2692,7 +2708,7 @@
       </c>
       <c r="BN14" t="inlineStr"/>
       <c r="BO14" t="n">
-        <v>0</v>
+        <v>4399570</v>
       </c>
       <c r="BP14" t="n">
         <v>0</v>
@@ -2703,10 +2719,14 @@
       <c r="BT14" t="n">
         <v>0</v>
       </c>
-      <c r="BU14" t="inlineStr"/>
+      <c r="BU14" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV14" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -2988,21 +3008,27 @@
       </c>
       <c r="BN16" t="inlineStr"/>
       <c r="BO16" t="n">
-        <v>0</v>
+        <v>27533660</v>
       </c>
       <c r="BP16" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ16" t="inlineStr"/>
+        <v>2160</v>
+      </c>
+      <c r="BQ16" t="n">
+        <v>12747.06</v>
+      </c>
       <c r="BR16" t="inlineStr"/>
       <c r="BS16" t="inlineStr"/>
       <c r="BT16" t="n">
         <v>0</v>
       </c>
-      <c r="BU16" t="inlineStr"/>
+      <c r="BU16" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV16" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -3564,7 +3590,7 @@
       </c>
       <c r="BN20" t="inlineStr"/>
       <c r="BO20" t="n">
-        <v>0</v>
+        <v>12195890</v>
       </c>
       <c r="BP20" t="n">
         <v>0</v>
@@ -3575,10 +3601,14 @@
       <c r="BT20" t="n">
         <v>0</v>
       </c>
-      <c r="BU20" t="inlineStr"/>
+      <c r="BU20" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV20" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -4280,7 +4310,7 @@
       </c>
       <c r="BN25" t="inlineStr"/>
       <c r="BO25" t="n">
-        <v>0</v>
+        <v>7815950</v>
       </c>
       <c r="BP25" t="n">
         <v>0</v>
@@ -4291,10 +4321,14 @@
       <c r="BT25" t="n">
         <v>0</v>
       </c>
-      <c r="BU25" t="inlineStr"/>
+      <c r="BU25" t="inlineStr">
+        <is>
+          <t>富邦</t>
+        </is>
+      </c>
       <c r="BV25" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -4436,21 +4470,27 @@
       </c>
       <c r="BN26" t="inlineStr"/>
       <c r="BO26" t="n">
-        <v>0</v>
+        <v>8294530</v>
       </c>
       <c r="BP26" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ26" t="inlineStr"/>
+        <v>2500</v>
+      </c>
+      <c r="BQ26" t="n">
+        <v>3317.81</v>
+      </c>
       <c r="BR26" t="inlineStr"/>
       <c r="BS26" t="inlineStr"/>
       <c r="BT26" t="n">
         <v>0</v>
       </c>
-      <c r="BU26" t="inlineStr"/>
+      <c r="BU26" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV26" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -4872,7 +4912,7 @@
       </c>
       <c r="BN29" t="inlineStr"/>
       <c r="BO29" t="n">
-        <v>0</v>
+        <v>24533050</v>
       </c>
       <c r="BP29" t="n">
         <v>0</v>
@@ -4883,10 +4923,14 @@
       <c r="BT29" t="n">
         <v>0</v>
       </c>
-      <c r="BU29" t="inlineStr"/>
+      <c r="BU29" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV29" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5072,7 @@
       </c>
       <c r="BN30" t="inlineStr"/>
       <c r="BO30" t="n">
-        <v>0</v>
+        <v>7317650</v>
       </c>
       <c r="BP30" t="n">
         <v>0</v>
@@ -5039,10 +5083,14 @@
       <c r="BT30" t="n">
         <v>0</v>
       </c>
-      <c r="BU30" t="inlineStr"/>
+      <c r="BU30" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV30" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -5736,7 +5784,7 @@
       </c>
       <c r="BN35" t="inlineStr"/>
       <c r="BO35" t="n">
-        <v>0</v>
+        <v>3928020</v>
       </c>
       <c r="BP35" t="n">
         <v>0</v>
@@ -5747,10 +5795,14 @@
       <c r="BT35" t="n">
         <v>0</v>
       </c>
-      <c r="BU35" t="inlineStr"/>
+      <c r="BU35" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV35" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -5890,21 +5942,27 @@
       </c>
       <c r="BN36" t="inlineStr"/>
       <c r="BO36" t="n">
-        <v>0</v>
+        <v>111096700</v>
       </c>
       <c r="BP36" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ36" t="inlineStr"/>
+        <v>2356440</v>
+      </c>
+      <c r="BQ36" t="n">
+        <v>47.15</v>
+      </c>
       <c r="BR36" t="inlineStr"/>
       <c r="BS36" t="inlineStr"/>
       <c r="BT36" t="n">
         <v>0</v>
       </c>
-      <c r="BU36" t="inlineStr"/>
+      <c r="BU36" t="inlineStr">
+        <is>
+          <t>台新</t>
+        </is>
+      </c>
       <c r="BV36" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -6044,7 +6102,7 @@
       </c>
       <c r="BN37" t="inlineStr"/>
       <c r="BO37" t="n">
-        <v>0</v>
+        <v>10995170</v>
       </c>
       <c r="BP37" t="n">
         <v>0</v>
@@ -6055,10 +6113,14 @@
       <c r="BT37" t="n">
         <v>0</v>
       </c>
-      <c r="BU37" t="inlineStr"/>
+      <c r="BU37" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV37" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -6198,7 +6260,7 @@
       </c>
       <c r="BN38" t="inlineStr"/>
       <c r="BO38" t="n">
-        <v>0</v>
+        <v>4346590</v>
       </c>
       <c r="BP38" t="n">
         <v>0</v>
@@ -6209,10 +6271,14 @@
       <c r="BT38" t="n">
         <v>0</v>
       </c>
-      <c r="BU38" t="inlineStr"/>
+      <c r="BU38" t="inlineStr">
+        <is>
+          <t>統一</t>
+        </is>
+      </c>
       <c r="BV38" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -6494,7 +6560,7 @@
       </c>
       <c r="BN40" t="inlineStr"/>
       <c r="BO40" t="n">
-        <v>0</v>
+        <v>21086550</v>
       </c>
       <c r="BP40" t="n">
         <v>0</v>
@@ -6505,10 +6571,14 @@
       <c r="BT40" t="n">
         <v>0</v>
       </c>
-      <c r="BU40" t="inlineStr"/>
+      <c r="BU40" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV40" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -6650,21 +6720,27 @@
       </c>
       <c r="BN41" t="inlineStr"/>
       <c r="BO41" t="n">
-        <v>0</v>
+        <v>23015150</v>
       </c>
       <c r="BP41" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ41" t="inlineStr"/>
+        <v>17920</v>
+      </c>
+      <c r="BQ41" t="n">
+        <v>1284.33</v>
+      </c>
       <c r="BR41" t="inlineStr"/>
       <c r="BS41" t="inlineStr"/>
       <c r="BT41" t="n">
         <v>0</v>
       </c>
-      <c r="BU41" t="inlineStr"/>
+      <c r="BU41" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV41" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -6806,7 +6882,7 @@
       </c>
       <c r="BN42" t="inlineStr"/>
       <c r="BO42" t="n">
-        <v>0</v>
+        <v>22794310</v>
       </c>
       <c r="BP42" t="n">
         <v>0</v>
@@ -6817,10 +6893,14 @@
       <c r="BT42" t="n">
         <v>0</v>
       </c>
-      <c r="BU42" t="inlineStr"/>
+      <c r="BU42" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV42" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -7102,21 +7182,27 @@
       </c>
       <c r="BN44" t="inlineStr"/>
       <c r="BO44" t="n">
-        <v>0</v>
+        <v>14647410</v>
       </c>
       <c r="BP44" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ44" t="inlineStr"/>
+        <v>112610</v>
+      </c>
+      <c r="BQ44" t="n">
+        <v>130.07</v>
+      </c>
       <c r="BR44" t="inlineStr"/>
       <c r="BS44" t="inlineStr"/>
       <c r="BT44" t="n">
         <v>0</v>
       </c>
-      <c r="BU44" t="inlineStr"/>
+      <c r="BU44" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV44" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -7398,21 +7484,27 @@
       </c>
       <c r="BN46" t="inlineStr"/>
       <c r="BO46" t="n">
-        <v>0</v>
+        <v>21235500</v>
       </c>
       <c r="BP46" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ46" t="inlineStr"/>
+        <v>97700</v>
+      </c>
+      <c r="BQ46" t="n">
+        <v>217.35</v>
+      </c>
       <c r="BR46" t="inlineStr"/>
       <c r="BS46" t="inlineStr"/>
       <c r="BT46" t="n">
         <v>0</v>
       </c>
-      <c r="BU46" t="inlineStr"/>
+      <c r="BU46" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV46" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -7554,7 +7646,7 @@
       </c>
       <c r="BN47" t="inlineStr"/>
       <c r="BO47" t="n">
-        <v>0</v>
+        <v>412690</v>
       </c>
       <c r="BP47" t="n">
         <v>0</v>
@@ -7565,10 +7657,14 @@
       <c r="BT47" t="n">
         <v>0</v>
       </c>
-      <c r="BU47" t="inlineStr"/>
+      <c r="BU47" t="inlineStr">
+        <is>
+          <t>國泰</t>
+        </is>
+      </c>
       <c r="BV47" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -7850,7 +7946,7 @@
       </c>
       <c r="BN49" t="inlineStr"/>
       <c r="BO49" t="n">
-        <v>0</v>
+        <v>20297100</v>
       </c>
       <c r="BP49" t="n">
         <v>0</v>
@@ -7861,10 +7957,14 @@
       <c r="BT49" t="n">
         <v>0</v>
       </c>
-      <c r="BU49" t="inlineStr"/>
+      <c r="BU49" t="inlineStr">
+        <is>
+          <t>群益</t>
+        </is>
+      </c>
       <c r="BV49" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -8146,21 +8246,27 @@
       </c>
       <c r="BN51" t="inlineStr"/>
       <c r="BO51" t="n">
-        <v>0</v>
+        <v>22554130</v>
       </c>
       <c r="BP51" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ51" t="inlineStr"/>
+        <v>134440</v>
+      </c>
+      <c r="BQ51" t="n">
+        <v>167.76</v>
+      </c>
       <c r="BR51" t="inlineStr"/>
       <c r="BS51" t="inlineStr"/>
       <c r="BT51" t="n">
         <v>0</v>
       </c>
-      <c r="BU51" t="inlineStr"/>
+      <c r="BU51" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV51" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -8302,7 +8408,7 @@
       </c>
       <c r="BN52" t="inlineStr"/>
       <c r="BO52" t="n">
-        <v>0</v>
+        <v>742620</v>
       </c>
       <c r="BP52" t="n">
         <v>0</v>
@@ -8313,10 +8419,14 @@
       <c r="BT52" t="n">
         <v>0</v>
       </c>
-      <c r="BU52" t="inlineStr"/>
+      <c r="BU52" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV52" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -9158,7 +9268,7 @@
       </c>
       <c r="BN58" t="inlineStr"/>
       <c r="BO58" t="n">
-        <v>0</v>
+        <v>1074970</v>
       </c>
       <c r="BP58" t="n">
         <v>0</v>
@@ -9169,10 +9279,14 @@
       <c r="BT58" t="n">
         <v>0</v>
       </c>
-      <c r="BU58" t="inlineStr"/>
+      <c r="BU58" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV58" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -10712,7 +10826,7 @@
       </c>
       <c r="BN69" t="inlineStr"/>
       <c r="BO69" t="n">
-        <v>0</v>
+        <v>4432990</v>
       </c>
       <c r="BP69" t="n">
         <v>0</v>
@@ -10723,10 +10837,14 @@
       <c r="BT69" t="n">
         <v>0</v>
       </c>
-      <c r="BU69" t="inlineStr"/>
+      <c r="BU69" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV69" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -12330,7 +12448,7 @@
       </c>
       <c r="BN80" t="inlineStr"/>
       <c r="BO80" t="n">
-        <v>0</v>
+        <v>8504380</v>
       </c>
       <c r="BP80" t="n">
         <v>0</v>
@@ -12341,10 +12459,14 @@
       <c r="BT80" t="n">
         <v>0</v>
       </c>
-      <c r="BU80" t="inlineStr"/>
+      <c r="BU80" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV80" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -12568,7 +12690,7 @@
       </c>
       <c r="BN81" t="inlineStr"/>
       <c r="BO81" t="n">
-        <v>0</v>
+        <v>822090</v>
       </c>
       <c r="BP81" t="n">
         <v>0</v>
@@ -12579,10 +12701,14 @@
       <c r="BT81" t="n">
         <v>0</v>
       </c>
-      <c r="BU81" t="inlineStr"/>
+      <c r="BU81" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV81" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -12806,7 +12932,7 @@
       </c>
       <c r="BN82" t="inlineStr"/>
       <c r="BO82" t="n">
-        <v>0</v>
+        <v>4361860</v>
       </c>
       <c r="BP82" t="n">
         <v>0</v>
@@ -12817,10 +12943,14 @@
       <c r="BT82" t="n">
         <v>0</v>
       </c>
-      <c r="BU82" t="inlineStr"/>
+      <c r="BU82" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV82" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -13044,21 +13174,27 @@
       </c>
       <c r="BN83" t="inlineStr"/>
       <c r="BO83" t="n">
-        <v>0</v>
+        <v>13728580</v>
       </c>
       <c r="BP83" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ83" t="inlineStr"/>
+        <v>456310</v>
+      </c>
+      <c r="BQ83" t="n">
+        <v>30.09</v>
+      </c>
       <c r="BR83" t="inlineStr"/>
       <c r="BS83" t="inlineStr"/>
       <c r="BT83" t="n">
         <v>0</v>
       </c>
-      <c r="BU83" t="inlineStr"/>
+      <c r="BU83" t="inlineStr">
+        <is>
+          <t>群益</t>
+        </is>
+      </c>
       <c r="BV83" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -13282,7 +13418,7 @@
       </c>
       <c r="BN84" t="inlineStr"/>
       <c r="BO84" t="n">
-        <v>0</v>
+        <v>20066610</v>
       </c>
       <c r="BP84" t="n">
         <v>0</v>
@@ -13293,10 +13429,14 @@
       <c r="BT84" t="n">
         <v>0</v>
       </c>
-      <c r="BU84" t="inlineStr"/>
+      <c r="BU84" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV84" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -13520,21 +13660,27 @@
       </c>
       <c r="BN85" t="inlineStr"/>
       <c r="BO85" t="n">
-        <v>0</v>
+        <v>6760120</v>
       </c>
       <c r="BP85" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ85" t="inlineStr"/>
+        <v>1050</v>
+      </c>
+      <c r="BQ85" t="n">
+        <v>6438.21</v>
+      </c>
       <c r="BR85" t="inlineStr"/>
       <c r="BS85" t="inlineStr"/>
       <c r="BT85" t="n">
         <v>0</v>
       </c>
-      <c r="BU85" t="inlineStr"/>
+      <c r="BU85" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV85" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -14202,7 +14348,7 @@
       </c>
       <c r="BN88" t="inlineStr"/>
       <c r="BO88" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="BP88" t="n">
         <v>0</v>
@@ -14213,10 +14359,14 @@
       <c r="BT88" t="n">
         <v>0</v>
       </c>
-      <c r="BU88" t="inlineStr"/>
+      <c r="BU88" t="inlineStr">
+        <is>
+          <t>兆豐</t>
+        </is>
+      </c>
       <c r="BV88" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -14440,7 +14590,7 @@
       </c>
       <c r="BN89" t="inlineStr"/>
       <c r="BO89" t="n">
-        <v>0</v>
+        <v>28530</v>
       </c>
       <c r="BP89" t="n">
         <v>0</v>
@@ -14451,10 +14601,14 @@
       <c r="BT89" t="n">
         <v>0</v>
       </c>
-      <c r="BU89" t="inlineStr"/>
+      <c r="BU89" t="inlineStr">
+        <is>
+          <t>國泰</t>
+        </is>
+      </c>
       <c r="BV89" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -15122,7 +15276,7 @@
       </c>
       <c r="BN92" t="inlineStr"/>
       <c r="BO92" t="n">
-        <v>0</v>
+        <v>8047800</v>
       </c>
       <c r="BP92" t="n">
         <v>0</v>
@@ -15133,10 +15287,14 @@
       <c r="BT92" t="n">
         <v>0</v>
       </c>
-      <c r="BU92" t="inlineStr"/>
+      <c r="BU92" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV92" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -15364,21 +15522,27 @@
       </c>
       <c r="BN93" t="inlineStr"/>
       <c r="BO93" t="n">
-        <v>0</v>
+        <v>9053860</v>
       </c>
       <c r="BP93" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ93" t="inlineStr"/>
+        <v>189820</v>
+      </c>
+      <c r="BQ93" t="n">
+        <v>47.7</v>
+      </c>
       <c r="BR93" t="inlineStr"/>
       <c r="BS93" t="inlineStr"/>
       <c r="BT93" t="n">
         <v>0</v>
       </c>
-      <c r="BU93" t="inlineStr"/>
+      <c r="BU93" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV93" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -15606,21 +15770,27 @@
       </c>
       <c r="BN94" t="inlineStr"/>
       <c r="BO94" t="n">
-        <v>0</v>
+        <v>67969770</v>
       </c>
       <c r="BP94" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ94" t="inlineStr"/>
+        <v>84510</v>
+      </c>
+      <c r="BQ94" t="n">
+        <v>804.28</v>
+      </c>
       <c r="BR94" t="inlineStr"/>
       <c r="BS94" t="inlineStr"/>
       <c r="BT94" t="n">
         <v>0</v>
       </c>
-      <c r="BU94" t="inlineStr"/>
+      <c r="BU94" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV94" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -16070,7 +16240,7 @@
       </c>
       <c r="BN96" t="inlineStr"/>
       <c r="BO96" t="n">
-        <v>0</v>
+        <v>102470</v>
       </c>
       <c r="BP96" t="n">
         <v>0</v>
@@ -16081,10 +16251,14 @@
       <c r="BT96" t="n">
         <v>0</v>
       </c>
-      <c r="BU96" t="inlineStr"/>
+      <c r="BU96" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV96" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -16312,7 +16486,7 @@
       </c>
       <c r="BN97" t="inlineStr"/>
       <c r="BO97" t="n">
-        <v>0</v>
+        <v>5953770</v>
       </c>
       <c r="BP97" t="n">
         <v>0</v>
@@ -16323,10 +16497,14 @@
       <c r="BT97" t="n">
         <v>0</v>
       </c>
-      <c r="BU97" t="inlineStr"/>
+      <c r="BU97" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV97" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -16780,21 +16958,27 @@
       </c>
       <c r="BN99" t="inlineStr"/>
       <c r="BO99" t="n">
-        <v>0</v>
+        <v>23537930</v>
       </c>
       <c r="BP99" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ99" t="inlineStr"/>
+        <v>22850</v>
+      </c>
+      <c r="BQ99" t="n">
+        <v>1030.11</v>
+      </c>
       <c r="BR99" t="inlineStr"/>
       <c r="BS99" t="inlineStr"/>
       <c r="BT99" t="n">
         <v>0</v>
       </c>
-      <c r="BU99" t="inlineStr"/>
+      <c r="BU99" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV99" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -17022,21 +17206,27 @@
       </c>
       <c r="BN100" t="inlineStr"/>
       <c r="BO100" t="n">
-        <v>0</v>
+        <v>21479790</v>
       </c>
       <c r="BP100" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ100" t="inlineStr"/>
+        <v>6680</v>
+      </c>
+      <c r="BQ100" t="n">
+        <v>3215.54</v>
+      </c>
       <c r="BR100" t="inlineStr"/>
       <c r="BS100" t="inlineStr"/>
       <c r="BT100" t="n">
         <v>0</v>
       </c>
-      <c r="BU100" t="inlineStr"/>
+      <c r="BU100" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV100" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -17400,21 +17590,27 @@
       </c>
       <c r="BN102" t="inlineStr"/>
       <c r="BO102" t="n">
-        <v>0</v>
+        <v>6259170</v>
       </c>
       <c r="BP102" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ102" t="inlineStr"/>
+        <v>145780</v>
+      </c>
+      <c r="BQ102" t="n">
+        <v>42.94</v>
+      </c>
       <c r="BR102" t="inlineStr"/>
       <c r="BS102" t="inlineStr"/>
       <c r="BT102" t="n">
         <v>0</v>
       </c>
-      <c r="BU102" t="inlineStr"/>
+      <c r="BU102" t="inlineStr">
+        <is>
+          <t>兆豐</t>
+        </is>
+      </c>
       <c r="BV102" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -17688,21 +17884,27 @@
       </c>
       <c r="BN104" t="inlineStr"/>
       <c r="BO104" t="n">
-        <v>0</v>
+        <v>9053860</v>
       </c>
       <c r="BP104" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ104" t="inlineStr"/>
+        <v>189820</v>
+      </c>
+      <c r="BQ104" t="n">
+        <v>47.7</v>
+      </c>
       <c r="BR104" t="inlineStr"/>
       <c r="BS104" t="inlineStr"/>
       <c r="BT104" t="n">
         <v>0</v>
       </c>
-      <c r="BU104" t="inlineStr"/>
+      <c r="BU104" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV104" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -18520,21 +18722,27 @@
       </c>
       <c r="BN110" t="inlineStr"/>
       <c r="BO110" t="n">
-        <v>0</v>
+        <v>21479790</v>
       </c>
       <c r="BP110" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ110" t="inlineStr"/>
+        <v>6680</v>
+      </c>
+      <c r="BQ110" t="n">
+        <v>3215.54</v>
+      </c>
       <c r="BR110" t="inlineStr"/>
       <c r="BS110" t="inlineStr"/>
       <c r="BT110" t="n">
         <v>0</v>
       </c>
-      <c r="BU110" t="inlineStr"/>
+      <c r="BU110" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV110" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -18944,21 +19152,27 @@
       </c>
       <c r="BN113" t="inlineStr"/>
       <c r="BO113" t="n">
-        <v>0</v>
+        <v>30260740</v>
       </c>
       <c r="BP113" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ113" t="inlineStr"/>
+        <v>5725560</v>
+      </c>
+      <c r="BQ113" t="n">
+        <v>5.29</v>
+      </c>
       <c r="BR113" t="inlineStr"/>
       <c r="BS113" t="inlineStr"/>
       <c r="BT113" t="n">
         <v>0</v>
       </c>
-      <c r="BU113" t="inlineStr"/>
+      <c r="BU113" t="inlineStr">
+        <is>
+          <t>群益</t>
+        </is>
+      </c>
       <c r="BV113" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -19096,21 +19310,27 @@
       </c>
       <c r="BN114" t="inlineStr"/>
       <c r="BO114" t="n">
-        <v>0</v>
+        <v>9478170</v>
       </c>
       <c r="BP114" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ114" t="inlineStr"/>
+        <v>20140</v>
+      </c>
+      <c r="BQ114" t="n">
+        <v>470.61</v>
+      </c>
       <c r="BR114" t="inlineStr"/>
       <c r="BS114" t="inlineStr"/>
       <c r="BT114" t="n">
         <v>0</v>
       </c>
-      <c r="BU114" t="inlineStr"/>
+      <c r="BU114" t="inlineStr">
+        <is>
+          <t>統一</t>
+        </is>
+      </c>
       <c r="BV114" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -19520,21 +19740,27 @@
       </c>
       <c r="BN117" t="inlineStr"/>
       <c r="BO117" t="n">
-        <v>0</v>
+        <v>7852990</v>
       </c>
       <c r="BP117" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ117" t="inlineStr"/>
+        <v>130</v>
+      </c>
+      <c r="BQ117" t="n">
+        <v>60407.62</v>
+      </c>
       <c r="BR117" t="inlineStr"/>
       <c r="BS117" t="inlineStr"/>
       <c r="BT117" t="n">
         <v>0</v>
       </c>
-      <c r="BU117" t="inlineStr"/>
+      <c r="BU117" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV117" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -19672,21 +19898,27 @@
       </c>
       <c r="BN118" t="inlineStr"/>
       <c r="BO118" t="n">
-        <v>0</v>
+        <v>2591890</v>
       </c>
       <c r="BP118" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ118" t="inlineStr"/>
+        <v>26900</v>
+      </c>
+      <c r="BQ118" t="n">
+        <v>96.34999999999999</v>
+      </c>
       <c r="BR118" t="inlineStr"/>
       <c r="BS118" t="inlineStr"/>
       <c r="BT118" t="n">
         <v>0</v>
       </c>
-      <c r="BU118" t="inlineStr"/>
+      <c r="BU118" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV118" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -19960,21 +20192,27 @@
       </c>
       <c r="BN120" t="inlineStr"/>
       <c r="BO120" t="n">
-        <v>0</v>
+        <v>3068470</v>
       </c>
       <c r="BP120" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ120" t="inlineStr"/>
+        <v>1950</v>
+      </c>
+      <c r="BQ120" t="n">
+        <v>1573.57</v>
+      </c>
       <c r="BR120" t="inlineStr"/>
       <c r="BS120" t="inlineStr"/>
       <c r="BT120" t="n">
         <v>0</v>
       </c>
-      <c r="BU120" t="inlineStr"/>
+      <c r="BU120" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV120" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -20112,21 +20350,27 @@
       </c>
       <c r="BN121" t="inlineStr"/>
       <c r="BO121" t="n">
-        <v>0</v>
+        <v>25964060</v>
       </c>
       <c r="BP121" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ121" t="inlineStr"/>
+        <v>222610</v>
+      </c>
+      <c r="BQ121" t="n">
+        <v>116.63</v>
+      </c>
       <c r="BR121" t="inlineStr"/>
       <c r="BS121" t="inlineStr"/>
       <c r="BT121" t="n">
         <v>0</v>
       </c>
-      <c r="BU121" t="inlineStr"/>
+      <c r="BU121" t="inlineStr">
+        <is>
+          <t>元富</t>
+        </is>
+      </c>
       <c r="BV121" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -20264,21 +20508,27 @@
       </c>
       <c r="BN122" t="inlineStr"/>
       <c r="BO122" t="n">
-        <v>0</v>
+        <v>1963740</v>
       </c>
       <c r="BP122" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ122" t="inlineStr"/>
+        <v>5200</v>
+      </c>
+      <c r="BQ122" t="n">
+        <v>377.64</v>
+      </c>
       <c r="BR122" t="inlineStr"/>
       <c r="BS122" t="inlineStr"/>
       <c r="BT122" t="n">
         <v>0</v>
       </c>
-      <c r="BU122" t="inlineStr"/>
+      <c r="BU122" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV122" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -20416,21 +20666,27 @@
       </c>
       <c r="BN123" t="inlineStr"/>
       <c r="BO123" t="n">
-        <v>0</v>
+        <v>24351970</v>
       </c>
       <c r="BP123" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ123" t="inlineStr"/>
+        <v>798830</v>
+      </c>
+      <c r="BQ123" t="n">
+        <v>30.48</v>
+      </c>
       <c r="BR123" t="inlineStr"/>
       <c r="BS123" t="inlineStr"/>
       <c r="BT123" t="n">
         <v>0</v>
       </c>
-      <c r="BU123" t="inlineStr"/>
+      <c r="BU123" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV123" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -20581,7 +20837,7 @@
       </c>
       <c r="BU124" t="inlineStr">
         <is>
-          <t>華南</t>
+          <t>中信</t>
         </is>
       </c>
       <c r="BV124" t="inlineStr">
@@ -20724,7 +20980,7 @@
       </c>
       <c r="BN125" t="inlineStr"/>
       <c r="BO125" t="n">
-        <v>0</v>
+        <v>1313240</v>
       </c>
       <c r="BP125" t="n">
         <v>0</v>
@@ -20735,10 +20991,14 @@
       <c r="BT125" t="n">
         <v>0</v>
       </c>
-      <c r="BU125" t="inlineStr"/>
+      <c r="BU125" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV125" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -20876,7 +21136,7 @@
       </c>
       <c r="BN126" t="inlineStr"/>
       <c r="BO126" t="n">
-        <v>0</v>
+        <v>3572240</v>
       </c>
       <c r="BP126" t="n">
         <v>0</v>
@@ -20887,10 +21147,14 @@
       <c r="BT126" t="n">
         <v>0</v>
       </c>
-      <c r="BU126" t="inlineStr"/>
+      <c r="BU126" t="inlineStr">
+        <is>
+          <t>永豐</t>
+        </is>
+      </c>
       <c r="BV126" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -21028,7 +21292,7 @@
       </c>
       <c r="BN127" t="inlineStr"/>
       <c r="BO127" t="n">
-        <v>0</v>
+        <v>852570</v>
       </c>
       <c r="BP127" t="n">
         <v>0</v>
@@ -21039,10 +21303,14 @@
       <c r="BT127" t="n">
         <v>0</v>
       </c>
-      <c r="BU127" t="inlineStr"/>
+      <c r="BU127" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV127" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -21180,21 +21448,27 @@
       </c>
       <c r="BN128" t="inlineStr"/>
       <c r="BO128" t="n">
-        <v>0</v>
+        <v>37425840</v>
       </c>
       <c r="BP128" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ128" t="inlineStr"/>
+        <v>1356510</v>
+      </c>
+      <c r="BQ128" t="n">
+        <v>27.59</v>
+      </c>
       <c r="BR128" t="inlineStr"/>
       <c r="BS128" t="inlineStr"/>
       <c r="BT128" t="n">
         <v>0</v>
       </c>
-      <c r="BU128" t="inlineStr"/>
+      <c r="BU128" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV128" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -21332,7 +21606,7 @@
       </c>
       <c r="BN129" t="inlineStr"/>
       <c r="BO129" t="n">
-        <v>0</v>
+        <v>1619890</v>
       </c>
       <c r="BP129" t="n">
         <v>0</v>
@@ -21343,10 +21617,14 @@
       <c r="BT129" t="n">
         <v>0</v>
       </c>
-      <c r="BU129" t="inlineStr"/>
+      <c r="BU129" t="inlineStr">
+        <is>
+          <t>台新</t>
+        </is>
+      </c>
       <c r="BV129" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -22502,21 +22780,27 @@
       </c>
       <c r="BN138" t="inlineStr"/>
       <c r="BO138" t="n">
-        <v>0</v>
+        <v>5329420</v>
       </c>
       <c r="BP138" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ138" t="inlineStr"/>
+        <v>1175500</v>
+      </c>
+      <c r="BQ138" t="n">
+        <v>4.53</v>
+      </c>
       <c r="BR138" t="inlineStr"/>
       <c r="BS138" t="inlineStr"/>
       <c r="BT138" t="n">
         <v>0</v>
       </c>
-      <c r="BU138" t="inlineStr"/>
+      <c r="BU138" t="inlineStr">
+        <is>
+          <t>統一</t>
+        </is>
+      </c>
       <c r="BV138" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -22770,21 +23054,27 @@
       </c>
       <c r="BN140" t="inlineStr"/>
       <c r="BO140" t="n">
-        <v>0</v>
+        <v>17038820</v>
       </c>
       <c r="BP140" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ140" t="inlineStr"/>
+        <v>208540</v>
+      </c>
+      <c r="BQ140" t="n">
+        <v>81.70999999999999</v>
+      </c>
       <c r="BR140" t="inlineStr"/>
       <c r="BS140" t="inlineStr"/>
       <c r="BT140" t="n">
         <v>0</v>
       </c>
-      <c r="BU140" t="inlineStr"/>
+      <c r="BU140" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV140" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -22912,21 +23202,27 @@
       </c>
       <c r="BN141" t="inlineStr"/>
       <c r="BO141" t="n">
-        <v>0</v>
+        <v>71088200</v>
       </c>
       <c r="BP141" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ141" t="inlineStr"/>
+        <v>3300080</v>
+      </c>
+      <c r="BQ141" t="n">
+        <v>21.54</v>
+      </c>
       <c r="BR141" t="inlineStr"/>
       <c r="BS141" t="inlineStr"/>
       <c r="BT141" t="n">
         <v>0</v>
       </c>
-      <c r="BU141" t="inlineStr"/>
+      <c r="BU141" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV141" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -23180,7 +23476,7 @@
       </c>
       <c r="BN143" t="inlineStr"/>
       <c r="BO143" t="n">
-        <v>0</v>
+        <v>431870</v>
       </c>
       <c r="BP143" t="n">
         <v>0</v>
@@ -23191,10 +23487,14 @@
       <c r="BT143" t="n">
         <v>0</v>
       </c>
-      <c r="BU143" t="inlineStr"/>
+      <c r="BU143" t="inlineStr">
+        <is>
+          <t>永豐</t>
+        </is>
+      </c>
       <c r="BV143" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -23448,7 +23748,7 @@
       </c>
       <c r="BN145" t="inlineStr"/>
       <c r="BO145" t="n">
-        <v>0</v>
+        <v>2746590</v>
       </c>
       <c r="BP145" t="n">
         <v>0</v>
@@ -23459,10 +23759,14 @@
       <c r="BT145" t="n">
         <v>0</v>
       </c>
-      <c r="BU145" t="inlineStr"/>
+      <c r="BU145" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV145" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -23590,7 +23894,7 @@
       </c>
       <c r="BN146" t="inlineStr"/>
       <c r="BO146" t="n">
-        <v>0</v>
+        <v>1490940</v>
       </c>
       <c r="BP146" t="n">
         <v>0</v>
@@ -23601,10 +23905,14 @@
       <c r="BT146" t="n">
         <v>0</v>
       </c>
-      <c r="BU146" t="inlineStr"/>
+      <c r="BU146" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV146" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -24614,21 +24922,27 @@
       </c>
       <c r="BN154" t="inlineStr"/>
       <c r="BO154" t="n">
-        <v>0</v>
+        <v>86240710</v>
       </c>
       <c r="BP154" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ154" t="inlineStr"/>
+        <v>1975260</v>
+      </c>
+      <c r="BQ154" t="n">
+        <v>43.66</v>
+      </c>
       <c r="BR154" t="inlineStr"/>
       <c r="BS154" t="inlineStr"/>
       <c r="BT154" t="n">
         <v>0</v>
       </c>
-      <c r="BU154" t="inlineStr"/>
+      <c r="BU154" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV154" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -24756,7 +25070,7 @@
       </c>
       <c r="BN155" t="inlineStr"/>
       <c r="BO155" t="n">
-        <v>0</v>
+        <v>2429280</v>
       </c>
       <c r="BP155" t="n">
         <v>0</v>
@@ -24774,7 +25088,7 @@
       </c>
       <c r="BV155" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -24902,21 +25216,27 @@
       </c>
       <c r="BN156" t="inlineStr"/>
       <c r="BO156" t="n">
-        <v>0</v>
+        <v>23537930</v>
       </c>
       <c r="BP156" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ156" t="inlineStr"/>
+        <v>22850</v>
+      </c>
+      <c r="BQ156" t="n">
+        <v>1030.11</v>
+      </c>
       <c r="BR156" t="inlineStr"/>
       <c r="BS156" t="inlineStr"/>
       <c r="BT156" t="n">
         <v>0</v>
       </c>
-      <c r="BU156" t="inlineStr"/>
+      <c r="BU156" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV156" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -25044,7 +25364,7 @@
       </c>
       <c r="BN157" t="inlineStr"/>
       <c r="BO157" t="n">
-        <v>0</v>
+        <v>167640</v>
       </c>
       <c r="BP157" t="n">
         <v>0</v>
@@ -25057,12 +25377,12 @@
       </c>
       <c r="BU157" t="inlineStr">
         <is>
-          <t>永豐</t>
+          <t>富邦</t>
         </is>
       </c>
       <c r="BV157" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -25190,7 +25510,7 @@
       </c>
       <c r="BN158" t="inlineStr"/>
       <c r="BO158" t="n">
-        <v>0</v>
+        <v>5976880</v>
       </c>
       <c r="BP158" t="n">
         <v>0</v>
@@ -25208,7 +25528,7 @@
       </c>
       <c r="BV158" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -25336,12 +25656,14 @@
       </c>
       <c r="BN159" t="inlineStr"/>
       <c r="BO159" t="n">
-        <v>0</v>
+        <v>3043900</v>
       </c>
       <c r="BP159" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ159" t="inlineStr"/>
+        <v>500</v>
+      </c>
+      <c r="BQ159" t="n">
+        <v>6087.8</v>
+      </c>
       <c r="BR159" t="inlineStr"/>
       <c r="BS159" t="inlineStr"/>
       <c r="BT159" t="n">
@@ -25349,12 +25671,12 @@
       </c>
       <c r="BU159" t="inlineStr">
         <is>
-          <t>國泰</t>
+          <t>富邦</t>
         </is>
       </c>
       <c r="BV159" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -25482,7 +25804,7 @@
       </c>
       <c r="BN160" t="inlineStr"/>
       <c r="BO160" t="n">
-        <v>0</v>
+        <v>2182560</v>
       </c>
       <c r="BP160" t="n">
         <v>0</v>
@@ -25500,7 +25822,7 @@
       </c>
       <c r="BV160" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -25628,7 +25950,7 @@
       </c>
       <c r="BN161" t="inlineStr"/>
       <c r="BO161" t="n">
-        <v>0</v>
+        <v>20066610</v>
       </c>
       <c r="BP161" t="n">
         <v>0</v>
@@ -25639,10 +25961,14 @@
       <c r="BT161" t="n">
         <v>0</v>
       </c>
-      <c r="BU161" t="inlineStr"/>
+      <c r="BU161" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV161" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -25770,21 +26096,27 @@
       </c>
       <c r="BN162" t="inlineStr"/>
       <c r="BO162" t="n">
-        <v>0</v>
+        <v>13728580</v>
       </c>
       <c r="BP162" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ162" t="inlineStr"/>
+        <v>456310</v>
+      </c>
+      <c r="BQ162" t="n">
+        <v>30.09</v>
+      </c>
       <c r="BR162" t="inlineStr"/>
       <c r="BS162" t="inlineStr"/>
       <c r="BT162" t="n">
         <v>0</v>
       </c>
-      <c r="BU162" t="inlineStr"/>
+      <c r="BU162" t="inlineStr">
+        <is>
+          <t>群益</t>
+        </is>
+      </c>
       <c r="BV162" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -26038,7 +26370,7 @@
       </c>
       <c r="BN164" t="inlineStr"/>
       <c r="BO164" t="n">
-        <v>0</v>
+        <v>122480</v>
       </c>
       <c r="BP164" t="n">
         <v>0</v>
@@ -26049,10 +26381,14 @@
       <c r="BT164" t="n">
         <v>0</v>
       </c>
-      <c r="BU164" t="inlineStr"/>
+      <c r="BU164" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV164" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -26180,7 +26516,7 @@
       </c>
       <c r="BN165" t="inlineStr"/>
       <c r="BO165" t="n">
-        <v>0</v>
+        <v>3984800</v>
       </c>
       <c r="BP165" t="n">
         <v>0</v>
@@ -26191,10 +26527,14 @@
       <c r="BT165" t="n">
         <v>0</v>
       </c>
-      <c r="BU165" t="inlineStr"/>
+      <c r="BU165" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV165" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -26322,21 +26662,27 @@
       </c>
       <c r="BN166" t="inlineStr"/>
       <c r="BO166" t="n">
-        <v>0</v>
+        <v>39452220</v>
       </c>
       <c r="BP166" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ166" t="inlineStr"/>
+        <v>28450</v>
+      </c>
+      <c r="BQ166" t="n">
+        <v>1386.72</v>
+      </c>
       <c r="BR166" t="inlineStr"/>
       <c r="BS166" t="inlineStr"/>
       <c r="BT166" t="n">
         <v>0</v>
       </c>
-      <c r="BU166" t="inlineStr"/>
+      <c r="BU166" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV166" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -26464,7 +26810,7 @@
       </c>
       <c r="BN167" t="inlineStr"/>
       <c r="BO167" t="n">
-        <v>0</v>
+        <v>5953770</v>
       </c>
       <c r="BP167" t="n">
         <v>0</v>
@@ -26475,10 +26821,14 @@
       <c r="BT167" t="n">
         <v>0</v>
       </c>
-      <c r="BU167" t="inlineStr"/>
+      <c r="BU167" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV167" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -26606,7 +26956,7 @@
       </c>
       <c r="BN168" t="inlineStr"/>
       <c r="BO168" t="n">
-        <v>0</v>
+        <v>822090</v>
       </c>
       <c r="BP168" t="n">
         <v>0</v>
@@ -26617,10 +26967,14 @@
       <c r="BT168" t="n">
         <v>0</v>
       </c>
-      <c r="BU168" t="inlineStr"/>
+      <c r="BU168" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV168" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -26748,21 +27102,27 @@
       </c>
       <c r="BN169" t="inlineStr"/>
       <c r="BO169" t="n">
-        <v>0</v>
+        <v>67969770</v>
       </c>
       <c r="BP169" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ169" t="inlineStr"/>
+        <v>84510</v>
+      </c>
+      <c r="BQ169" t="n">
+        <v>804.28</v>
+      </c>
       <c r="BR169" t="inlineStr"/>
       <c r="BS169" t="inlineStr"/>
       <c r="BT169" t="n">
         <v>0</v>
       </c>
-      <c r="BU169" t="inlineStr"/>
+      <c r="BU169" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV169" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -26890,21 +27250,27 @@
       </c>
       <c r="BN170" t="inlineStr"/>
       <c r="BO170" t="n">
-        <v>0</v>
+        <v>6760120</v>
       </c>
       <c r="BP170" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ170" t="inlineStr"/>
+        <v>1050</v>
+      </c>
+      <c r="BQ170" t="n">
+        <v>6438.21</v>
+      </c>
       <c r="BR170" t="inlineStr"/>
       <c r="BS170" t="inlineStr"/>
       <c r="BT170" t="n">
         <v>0</v>
       </c>
-      <c r="BU170" t="inlineStr"/>
+      <c r="BU170" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV170" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -27032,21 +27398,27 @@
       </c>
       <c r="BN171" t="inlineStr"/>
       <c r="BO171" t="n">
-        <v>0</v>
+        <v>16730930</v>
       </c>
       <c r="BP171" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ171" t="inlineStr"/>
+        <v>227300</v>
+      </c>
+      <c r="BQ171" t="n">
+        <v>73.61</v>
+      </c>
       <c r="BR171" t="inlineStr"/>
       <c r="BS171" t="inlineStr"/>
       <c r="BT171" t="n">
         <v>0</v>
       </c>
-      <c r="BU171" t="inlineStr"/>
+      <c r="BU171" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV171" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -27552,7 +27924,7 @@
       </c>
       <c r="BN175" t="inlineStr"/>
       <c r="BO175" t="n">
-        <v>0</v>
+        <v>34000</v>
       </c>
       <c r="BP175" t="n">
         <v>0</v>
@@ -27563,10 +27935,14 @@
       <c r="BT175" t="n">
         <v>0</v>
       </c>
-      <c r="BU175" t="inlineStr"/>
+      <c r="BU175" t="inlineStr">
+        <is>
+          <t>元富</t>
+        </is>
+      </c>
       <c r="BV175" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -27694,7 +28070,7 @@
       </c>
       <c r="BN176" t="inlineStr"/>
       <c r="BO176" t="n">
-        <v>0</v>
+        <v>8047800</v>
       </c>
       <c r="BP176" t="n">
         <v>0</v>
@@ -27705,10 +28081,14 @@
       <c r="BT176" t="n">
         <v>0</v>
       </c>
-      <c r="BU176" t="inlineStr"/>
+      <c r="BU176" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV176" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -27962,7 +28342,7 @@
       </c>
       <c r="BN178" t="inlineStr"/>
       <c r="BO178" t="n">
-        <v>0</v>
+        <v>2990060</v>
       </c>
       <c r="BP178" t="n">
         <v>0</v>
@@ -27973,10 +28353,14 @@
       <c r="BT178" t="n">
         <v>0</v>
       </c>
-      <c r="BU178" t="inlineStr"/>
+      <c r="BU178" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV178" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -28104,7 +28488,7 @@
       </c>
       <c r="BN179" t="inlineStr"/>
       <c r="BO179" t="n">
-        <v>0</v>
+        <v>28530</v>
       </c>
       <c r="BP179" t="n">
         <v>0</v>
@@ -28115,10 +28499,14 @@
       <c r="BT179" t="n">
         <v>0</v>
       </c>
-      <c r="BU179" t="inlineStr"/>
+      <c r="BU179" t="inlineStr">
+        <is>
+          <t>國泰</t>
+        </is>
+      </c>
       <c r="BV179" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -28372,7 +28760,7 @@
       </c>
       <c r="BN181" t="inlineStr"/>
       <c r="BO181" t="n">
-        <v>0</v>
+        <v>6944990</v>
       </c>
       <c r="BP181" t="n">
         <v>0</v>
@@ -28383,10 +28771,14 @@
       <c r="BT181" t="n">
         <v>0</v>
       </c>
-      <c r="BU181" t="inlineStr"/>
+      <c r="BU181" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV181" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -28527,7 +28919,7 @@
       </c>
       <c r="BU182" t="inlineStr">
         <is>
-          <t>國票</t>
+          <t>中信</t>
         </is>
       </c>
       <c r="BV182" t="inlineStr">
@@ -28912,7 +29304,7 @@
       </c>
       <c r="BN185" t="inlineStr"/>
       <c r="BO185" t="n">
-        <v>0</v>
+        <v>102470</v>
       </c>
       <c r="BP185" t="n">
         <v>0</v>
@@ -28923,10 +29315,14 @@
       <c r="BT185" t="n">
         <v>0</v>
       </c>
-      <c r="BU185" t="inlineStr"/>
+      <c r="BU185" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV185" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -29054,21 +29450,27 @@
       </c>
       <c r="BN186" t="inlineStr"/>
       <c r="BO186" t="n">
-        <v>0</v>
+        <v>11247950</v>
       </c>
       <c r="BP186" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ186" t="inlineStr"/>
+        <v>49320</v>
+      </c>
+      <c r="BQ186" t="n">
+        <v>228.06</v>
+      </c>
       <c r="BR186" t="inlineStr"/>
       <c r="BS186" t="inlineStr"/>
       <c r="BT186" t="n">
         <v>0</v>
       </c>
-      <c r="BU186" t="inlineStr"/>
+      <c r="BU186" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV186" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -29322,21 +29724,27 @@
       </c>
       <c r="BN188" t="inlineStr"/>
       <c r="BO188" t="n">
-        <v>0</v>
+        <v>3982860</v>
       </c>
       <c r="BP188" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ188" t="inlineStr"/>
+        <v>109700</v>
+      </c>
+      <c r="BQ188" t="n">
+        <v>36.31</v>
+      </c>
       <c r="BR188" t="inlineStr"/>
       <c r="BS188" t="inlineStr"/>
       <c r="BT188" t="n">
         <v>0</v>
       </c>
-      <c r="BU188" t="inlineStr"/>
+      <c r="BU188" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV188" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -29590,7 +29998,7 @@
       </c>
       <c r="BN190" t="inlineStr"/>
       <c r="BO190" t="n">
-        <v>0</v>
+        <v>690200</v>
       </c>
       <c r="BP190" t="n">
         <v>0</v>
@@ -29601,10 +30009,14 @@
       <c r="BT190" t="n">
         <v>0</v>
       </c>
-      <c r="BU190" t="inlineStr"/>
+      <c r="BU190" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV190" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -29732,7 +30144,7 @@
       </c>
       <c r="BN191" t="inlineStr"/>
       <c r="BO191" t="n">
-        <v>0</v>
+        <v>895210</v>
       </c>
       <c r="BP191" t="n">
         <v>0</v>
@@ -29743,10 +30155,14 @@
       <c r="BT191" t="n">
         <v>0</v>
       </c>
-      <c r="BU191" t="inlineStr"/>
+      <c r="BU191" t="inlineStr">
+        <is>
+          <t>群益</t>
+        </is>
+      </c>
       <c r="BV191" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -29874,21 +30290,27 @@
       </c>
       <c r="BN192" t="inlineStr"/>
       <c r="BO192" t="n">
-        <v>0</v>
+        <v>5519010</v>
       </c>
       <c r="BP192" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ192" t="inlineStr"/>
+        <v>18950</v>
+      </c>
+      <c r="BQ192" t="n">
+        <v>291.24</v>
+      </c>
       <c r="BR192" t="inlineStr"/>
       <c r="BS192" t="inlineStr"/>
       <c r="BT192" t="n">
         <v>0</v>
       </c>
-      <c r="BU192" t="inlineStr"/>
+      <c r="BU192" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV192" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -30394,21 +30816,27 @@
       </c>
       <c r="BN196" t="inlineStr"/>
       <c r="BO196" t="n">
-        <v>0</v>
+        <v>35451090</v>
       </c>
       <c r="BP196" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ196" t="inlineStr"/>
+        <v>808740</v>
+      </c>
+      <c r="BQ196" t="n">
+        <v>43.83</v>
+      </c>
       <c r="BR196" t="inlineStr"/>
       <c r="BS196" t="inlineStr"/>
       <c r="BT196" t="n">
         <v>0</v>
       </c>
-      <c r="BU196" t="inlineStr"/>
+      <c r="BU196" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV196" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -30788,21 +31216,27 @@
       </c>
       <c r="BN199" t="inlineStr"/>
       <c r="BO199" t="n">
-        <v>0</v>
+        <v>34408480</v>
       </c>
       <c r="BP199" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ199" t="inlineStr"/>
+        <v>1238330</v>
+      </c>
+      <c r="BQ199" t="n">
+        <v>27.79</v>
+      </c>
       <c r="BR199" t="inlineStr"/>
       <c r="BS199" t="inlineStr"/>
       <c r="BT199" t="n">
         <v>0</v>
       </c>
-      <c r="BU199" t="inlineStr"/>
+      <c r="BU199" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV199" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -30930,7 +31364,7 @@
       </c>
       <c r="BN200" t="inlineStr"/>
       <c r="BO200" t="n">
-        <v>0</v>
+        <v>12822110</v>
       </c>
       <c r="BP200" t="n">
         <v>0</v>
@@ -30943,12 +31377,12 @@
       </c>
       <c r="BU200" t="inlineStr">
         <is>
-          <t>中信</t>
+          <t>富邦</t>
         </is>
       </c>
       <c r="BV200" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -31076,7 +31510,7 @@
       </c>
       <c r="BN201" t="inlineStr"/>
       <c r="BO201" t="n">
-        <v>0</v>
+        <v>647590</v>
       </c>
       <c r="BP201" t="n">
         <v>0</v>
@@ -31089,12 +31523,12 @@
       </c>
       <c r="BU201" t="inlineStr">
         <is>
-          <t>兆豐</t>
+          <t>富邦</t>
         </is>
       </c>
       <c r="BV201" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -31233,7 +31667,11 @@
       <c r="BT202" t="n">
         <v>0</v>
       </c>
-      <c r="BU202" t="inlineStr"/>
+      <c r="BU202" t="inlineStr">
+        <is>
+          <t>元展</t>
+        </is>
+      </c>
       <c r="BV202" t="inlineStr">
         <is>
           <t>今日無可用權證成交金額</t>
@@ -31364,7 +31802,7 @@
       </c>
       <c r="BN203" t="inlineStr"/>
       <c r="BO203" t="n">
-        <v>0</v>
+        <v>4361860</v>
       </c>
       <c r="BP203" t="n">
         <v>0</v>
@@ -31375,10 +31813,14 @@
       <c r="BT203" t="n">
         <v>0</v>
       </c>
-      <c r="BU203" t="inlineStr"/>
+      <c r="BU203" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV203" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -31632,7 +32074,7 @@
       </c>
       <c r="BN205" t="inlineStr"/>
       <c r="BO205" t="n">
-        <v>0</v>
+        <v>606990</v>
       </c>
       <c r="BP205" t="n">
         <v>0</v>
@@ -31643,10 +32085,14 @@
       <c r="BT205" t="n">
         <v>0</v>
       </c>
-      <c r="BU205" t="inlineStr"/>
+      <c r="BU205" t="inlineStr">
+        <is>
+          <t>永豐</t>
+        </is>
+      </c>
       <c r="BV205" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -31774,21 +32220,27 @@
       </c>
       <c r="BN206" t="inlineStr"/>
       <c r="BO206" t="n">
-        <v>0</v>
+        <v>11232390</v>
       </c>
       <c r="BP206" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ206" t="inlineStr"/>
+        <v>45000</v>
+      </c>
+      <c r="BQ206" t="n">
+        <v>249.61</v>
+      </c>
       <c r="BR206" t="inlineStr"/>
       <c r="BS206" t="inlineStr"/>
       <c r="BT206" t="n">
         <v>0</v>
       </c>
-      <c r="BU206" t="inlineStr"/>
+      <c r="BU206" t="inlineStr">
+        <is>
+          <t>統一</t>
+        </is>
+      </c>
       <c r="BV206" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -32168,7 +32620,7 @@
       </c>
       <c r="BN209" t="inlineStr"/>
       <c r="BO209" t="n">
-        <v>0</v>
+        <v>8504380</v>
       </c>
       <c r="BP209" t="n">
         <v>0</v>
@@ -32179,10 +32631,14 @@
       <c r="BT209" t="n">
         <v>0</v>
       </c>
-      <c r="BU209" t="inlineStr"/>
+      <c r="BU209" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV209" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -32436,7 +32892,7 @@
       </c>
       <c r="BN211" t="inlineStr"/>
       <c r="BO211" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="BP211" t="n">
         <v>0</v>
@@ -32447,10 +32903,14 @@
       <c r="BT211" t="n">
         <v>0</v>
       </c>
-      <c r="BU211" t="inlineStr"/>
+      <c r="BU211" t="inlineStr">
+        <is>
+          <t>兆豐</t>
+        </is>
+      </c>
       <c r="BV211" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -33082,21 +33542,27 @@
       </c>
       <c r="BN216" t="inlineStr"/>
       <c r="BO216" t="n">
-        <v>0</v>
+        <v>4615210</v>
       </c>
       <c r="BP216" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ216" t="inlineStr"/>
+        <v>27320</v>
+      </c>
+      <c r="BQ216" t="n">
+        <v>168.93</v>
+      </c>
       <c r="BR216" t="inlineStr"/>
       <c r="BS216" t="inlineStr"/>
       <c r="BT216" t="n">
         <v>0</v>
       </c>
-      <c r="BU216" t="inlineStr"/>
+      <c r="BU216" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV216" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -33224,21 +33690,27 @@
       </c>
       <c r="BN217" t="inlineStr"/>
       <c r="BO217" t="n">
-        <v>0</v>
+        <v>6699310</v>
       </c>
       <c r="BP217" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ217" t="inlineStr"/>
+        <v>208820</v>
+      </c>
+      <c r="BQ217" t="n">
+        <v>32.08</v>
+      </c>
       <c r="BR217" t="inlineStr"/>
       <c r="BS217" t="inlineStr"/>
       <c r="BT217" t="n">
         <v>0</v>
       </c>
-      <c r="BU217" t="inlineStr"/>
+      <c r="BU217" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV217" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -33366,21 +33838,27 @@
       </c>
       <c r="BN218" t="inlineStr"/>
       <c r="BO218" t="n">
-        <v>0</v>
+        <v>39784560</v>
       </c>
       <c r="BP218" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ218" t="inlineStr"/>
+        <v>484040</v>
+      </c>
+      <c r="BQ218" t="n">
+        <v>82.19</v>
+      </c>
       <c r="BR218" t="inlineStr"/>
       <c r="BS218" t="inlineStr"/>
       <c r="BT218" t="n">
         <v>0</v>
       </c>
-      <c r="BU218" t="inlineStr"/>
+      <c r="BU218" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV218" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -33634,7 +34112,7 @@
       </c>
       <c r="BN220" t="inlineStr"/>
       <c r="BO220" t="n">
-        <v>0</v>
+        <v>99810</v>
       </c>
       <c r="BP220" t="n">
         <v>0</v>
@@ -33645,10 +34123,14 @@
       <c r="BT220" t="n">
         <v>0</v>
       </c>
-      <c r="BU220" t="inlineStr"/>
+      <c r="BU220" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV220" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -33776,7 +34258,7 @@
       </c>
       <c r="BN221" t="inlineStr"/>
       <c r="BO221" t="n">
-        <v>0</v>
+        <v>4169330</v>
       </c>
       <c r="BP221" t="n">
         <v>0</v>
@@ -33787,10 +34269,14 @@
       <c r="BT221" t="n">
         <v>0</v>
       </c>
-      <c r="BU221" t="inlineStr"/>
+      <c r="BU221" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV221" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -34044,7 +34530,7 @@
       </c>
       <c r="BN223" t="inlineStr"/>
       <c r="BO223" t="n">
-        <v>0</v>
+        <v>8243810</v>
       </c>
       <c r="BP223" t="n">
         <v>0</v>
@@ -34055,10 +34541,14 @@
       <c r="BT223" t="n">
         <v>0</v>
       </c>
-      <c r="BU223" t="inlineStr"/>
+      <c r="BU223" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV223" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -34186,7 +34676,7 @@
       </c>
       <c r="BN224" t="inlineStr"/>
       <c r="BO224" t="n">
-        <v>0</v>
+        <v>5607680</v>
       </c>
       <c r="BP224" t="n">
         <v>0</v>
@@ -34197,10 +34687,14 @@
       <c r="BT224" t="n">
         <v>0</v>
       </c>
-      <c r="BU224" t="inlineStr"/>
+      <c r="BU224" t="inlineStr">
+        <is>
+          <t>富邦</t>
+        </is>
+      </c>
       <c r="BV224" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -34706,7 +35200,7 @@
       </c>
       <c r="BN228" t="inlineStr"/>
       <c r="BO228" t="n">
-        <v>0</v>
+        <v>755410</v>
       </c>
       <c r="BP228" t="n">
         <v>0</v>
@@ -34717,10 +35211,14 @@
       <c r="BT228" t="n">
         <v>0</v>
       </c>
-      <c r="BU228" t="inlineStr"/>
+      <c r="BU228" t="inlineStr">
+        <is>
+          <t>群益</t>
+        </is>
+      </c>
       <c r="BV228" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -34848,21 +35346,27 @@
       </c>
       <c r="BN229" t="inlineStr"/>
       <c r="BO229" t="n">
-        <v>0</v>
+        <v>48046350</v>
       </c>
       <c r="BP229" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ229" t="inlineStr"/>
+        <v>1397880</v>
+      </c>
+      <c r="BQ229" t="n">
+        <v>34.37</v>
+      </c>
       <c r="BR229" t="inlineStr"/>
       <c r="BS229" t="inlineStr"/>
       <c r="BT229" t="n">
         <v>0</v>
       </c>
-      <c r="BU229" t="inlineStr"/>
+      <c r="BU229" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV229" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -34990,7 +35494,7 @@
       </c>
       <c r="BN230" t="inlineStr"/>
       <c r="BO230" t="n">
-        <v>0</v>
+        <v>3471640</v>
       </c>
       <c r="BP230" t="n">
         <v>0</v>
@@ -35001,10 +35505,14 @@
       <c r="BT230" t="n">
         <v>0</v>
       </c>
-      <c r="BU230" t="inlineStr"/>
+      <c r="BU230" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV230" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -35258,7 +35766,7 @@
       </c>
       <c r="BN232" t="inlineStr"/>
       <c r="BO232" t="n">
-        <v>0</v>
+        <v>19180</v>
       </c>
       <c r="BP232" t="n">
         <v>0</v>
@@ -35269,10 +35777,14 @@
       <c r="BT232" t="n">
         <v>0</v>
       </c>
-      <c r="BU232" t="inlineStr"/>
+      <c r="BU232" t="inlineStr">
+        <is>
+          <t>永豐</t>
+        </is>
+      </c>
       <c r="BV232" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -35400,21 +35912,27 @@
       </c>
       <c r="BN233" t="inlineStr"/>
       <c r="BO233" t="n">
-        <v>0</v>
+        <v>12247650</v>
       </c>
       <c r="BP233" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ233" t="inlineStr"/>
+        <v>33810</v>
+      </c>
+      <c r="BQ233" t="n">
+        <v>362.25</v>
+      </c>
       <c r="BR233" t="inlineStr"/>
       <c r="BS233" t="inlineStr"/>
       <c r="BT233" t="n">
         <v>0</v>
       </c>
-      <c r="BU233" t="inlineStr"/>
+      <c r="BU233" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV233" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -35542,7 +36060,7 @@
       </c>
       <c r="BN234" t="inlineStr"/>
       <c r="BO234" t="n">
-        <v>0</v>
+        <v>3381580</v>
       </c>
       <c r="BP234" t="n">
         <v>0</v>
@@ -35553,10 +36071,14 @@
       <c r="BT234" t="n">
         <v>0</v>
       </c>
-      <c r="BU234" t="inlineStr"/>
+      <c r="BU234" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV234" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -35684,21 +36206,27 @@
       </c>
       <c r="BN235" t="inlineStr"/>
       <c r="BO235" t="n">
-        <v>0</v>
+        <v>1641030</v>
       </c>
       <c r="BP235" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ235" t="inlineStr"/>
+        <v>19500</v>
+      </c>
+      <c r="BQ235" t="n">
+        <v>84.16</v>
+      </c>
       <c r="BR235" t="inlineStr"/>
       <c r="BS235" t="inlineStr"/>
       <c r="BT235" t="n">
         <v>0</v>
       </c>
-      <c r="BU235" t="inlineStr"/>
+      <c r="BU235" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV235" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -35826,21 +36354,27 @@
       </c>
       <c r="BN236" t="inlineStr"/>
       <c r="BO236" t="n">
-        <v>0</v>
+        <v>17931910</v>
       </c>
       <c r="BP236" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ236" t="inlineStr"/>
+        <v>162130</v>
+      </c>
+      <c r="BQ236" t="n">
+        <v>110.6</v>
+      </c>
       <c r="BR236" t="inlineStr"/>
       <c r="BS236" t="inlineStr"/>
       <c r="BT236" t="n">
         <v>0</v>
       </c>
-      <c r="BU236" t="inlineStr"/>
+      <c r="BU236" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV236" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -35968,7 +36502,7 @@
       </c>
       <c r="BN237" t="inlineStr"/>
       <c r="BO237" t="n">
-        <v>0</v>
+        <v>758780</v>
       </c>
       <c r="BP237" t="n">
         <v>0</v>
@@ -35981,12 +36515,12 @@
       </c>
       <c r="BU237" t="inlineStr">
         <is>
-          <t>第一</t>
+          <t>群益</t>
         </is>
       </c>
       <c r="BV237" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -36114,21 +36648,27 @@
       </c>
       <c r="BN238" t="inlineStr"/>
       <c r="BO238" t="n">
-        <v>0</v>
+        <v>18727980</v>
       </c>
       <c r="BP238" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ238" t="inlineStr"/>
+        <v>1244270</v>
+      </c>
+      <c r="BQ238" t="n">
+        <v>15.05</v>
+      </c>
       <c r="BR238" t="inlineStr"/>
       <c r="BS238" t="inlineStr"/>
       <c r="BT238" t="n">
         <v>0</v>
       </c>
-      <c r="BU238" t="inlineStr"/>
+      <c r="BU238" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV238" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -36256,21 +36796,27 @@
       </c>
       <c r="BN239" t="inlineStr"/>
       <c r="BO239" t="n">
-        <v>0</v>
+        <v>59325140</v>
       </c>
       <c r="BP239" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ239" t="inlineStr"/>
+        <v>2835870</v>
+      </c>
+      <c r="BQ239" t="n">
+        <v>20.92</v>
+      </c>
       <c r="BR239" t="inlineStr"/>
       <c r="BS239" t="inlineStr"/>
       <c r="BT239" t="n">
         <v>0</v>
       </c>
-      <c r="BU239" t="inlineStr"/>
+      <c r="BU239" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV239" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -36398,21 +36944,27 @@
       </c>
       <c r="BN240" t="inlineStr"/>
       <c r="BO240" t="n">
-        <v>0</v>
+        <v>31007840</v>
       </c>
       <c r="BP240" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ240" t="inlineStr"/>
+        <v>1408320</v>
+      </c>
+      <c r="BQ240" t="n">
+        <v>22.02</v>
+      </c>
       <c r="BR240" t="inlineStr"/>
       <c r="BS240" t="inlineStr"/>
       <c r="BT240" t="n">
         <v>0</v>
       </c>
-      <c r="BU240" t="inlineStr"/>
+      <c r="BU240" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV240" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -36540,21 +37092,27 @@
       </c>
       <c r="BN241" t="inlineStr"/>
       <c r="BO241" t="n">
-        <v>0</v>
+        <v>57315210</v>
       </c>
       <c r="BP241" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ241" t="inlineStr"/>
+        <v>1156870</v>
+      </c>
+      <c r="BQ241" t="n">
+        <v>49.54</v>
+      </c>
       <c r="BR241" t="inlineStr"/>
       <c r="BS241" t="inlineStr"/>
       <c r="BT241" t="n">
         <v>0</v>
       </c>
-      <c r="BU241" t="inlineStr"/>
+      <c r="BU241" t="inlineStr">
+        <is>
+          <t>富邦</t>
+        </is>
+      </c>
       <c r="BV241" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -36682,7 +37240,7 @@
       </c>
       <c r="BN242" t="inlineStr"/>
       <c r="BO242" t="n">
-        <v>0</v>
+        <v>142050</v>
       </c>
       <c r="BP242" t="n">
         <v>0</v>
@@ -36695,12 +37253,12 @@
       </c>
       <c r="BU242" t="inlineStr">
         <is>
-          <t>玉山</t>
+          <t>富邦</t>
         </is>
       </c>
       <c r="BV242" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -36828,21 +37386,27 @@
       </c>
       <c r="BN243" t="inlineStr"/>
       <c r="BO243" t="n">
-        <v>0</v>
+        <v>9711960</v>
       </c>
       <c r="BP243" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ243" t="inlineStr"/>
+        <v>323710</v>
+      </c>
+      <c r="BQ243" t="n">
+        <v>30</v>
+      </c>
       <c r="BR243" t="inlineStr"/>
       <c r="BS243" t="inlineStr"/>
       <c r="BT243" t="n">
         <v>0</v>
       </c>
-      <c r="BU243" t="inlineStr"/>
+      <c r="BU243" t="inlineStr">
+        <is>
+          <t>永豐</t>
+        </is>
+      </c>
       <c r="BV243" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -36970,21 +37534,27 @@
       </c>
       <c r="BN244" t="inlineStr"/>
       <c r="BO244" t="n">
-        <v>0</v>
+        <v>14703320</v>
       </c>
       <c r="BP244" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ244" t="inlineStr"/>
+        <v>9800</v>
+      </c>
+      <c r="BQ244" t="n">
+        <v>1500.34</v>
+      </c>
       <c r="BR244" t="inlineStr"/>
       <c r="BS244" t="inlineStr"/>
       <c r="BT244" t="n">
         <v>0</v>
       </c>
-      <c r="BU244" t="inlineStr"/>
+      <c r="BU244" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV244" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -37112,21 +37682,27 @@
       </c>
       <c r="BN245" t="inlineStr"/>
       <c r="BO245" t="n">
-        <v>0</v>
+        <v>14002820</v>
       </c>
       <c r="BP245" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ245" t="inlineStr"/>
+        <v>114600</v>
+      </c>
+      <c r="BQ245" t="n">
+        <v>122.19</v>
+      </c>
       <c r="BR245" t="inlineStr"/>
       <c r="BS245" t="inlineStr"/>
       <c r="BT245" t="n">
         <v>0</v>
       </c>
-      <c r="BU245" t="inlineStr"/>
+      <c r="BU245" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV245" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -37517,7 +38093,11 @@
       <c r="BT248" t="n">
         <v>0</v>
       </c>
-      <c r="BU248" t="inlineStr"/>
+      <c r="BU248" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV248" t="inlineStr">
         <is>
           <t>今日無可用權證成交金額</t>
@@ -37900,7 +38480,7 @@
       </c>
       <c r="BN251" t="inlineStr"/>
       <c r="BO251" t="n">
-        <v>0</v>
+        <v>2364590</v>
       </c>
       <c r="BP251" t="n">
         <v>0</v>
@@ -37911,10 +38491,14 @@
       <c r="BT251" t="n">
         <v>0</v>
       </c>
-      <c r="BU251" t="inlineStr"/>
+      <c r="BU251" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV251" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -38294,7 +38878,7 @@
       </c>
       <c r="BN254" t="inlineStr"/>
       <c r="BO254" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="BP254" t="n">
         <v>0</v>
@@ -38305,10 +38889,14 @@
       <c r="BT254" t="n">
         <v>0</v>
       </c>
-      <c r="BU254" t="inlineStr"/>
+      <c r="BU254" t="inlineStr">
+        <is>
+          <t>永豐</t>
+        </is>
+      </c>
       <c r="BV254" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -38436,7 +39024,7 @@
       </c>
       <c r="BN255" t="inlineStr"/>
       <c r="BO255" t="n">
-        <v>0</v>
+        <v>1984450</v>
       </c>
       <c r="BP255" t="n">
         <v>0</v>
@@ -38447,10 +39035,14 @@
       <c r="BT255" t="n">
         <v>0</v>
       </c>
-      <c r="BU255" t="inlineStr"/>
+      <c r="BU255" t="inlineStr">
+        <is>
+          <t>永豐</t>
+        </is>
+      </c>
       <c r="BV255" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -38704,7 +39296,7 @@
       </c>
       <c r="BN257" t="inlineStr"/>
       <c r="BO257" t="n">
-        <v>0</v>
+        <v>6523450</v>
       </c>
       <c r="BP257" t="n">
         <v>0</v>
@@ -38715,10 +39307,14 @@
       <c r="BT257" t="n">
         <v>0</v>
       </c>
-      <c r="BU257" t="inlineStr"/>
+      <c r="BU257" t="inlineStr">
+        <is>
+          <t>統一</t>
+        </is>
+      </c>
       <c r="BV257" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -39350,7 +39946,7 @@
       </c>
       <c r="BN262" t="inlineStr"/>
       <c r="BO262" t="n">
-        <v>0</v>
+        <v>624700</v>
       </c>
       <c r="BP262" t="n">
         <v>0</v>
@@ -39361,10 +39957,14 @@
       <c r="BT262" t="n">
         <v>0</v>
       </c>
-      <c r="BU262" t="inlineStr"/>
+      <c r="BU262" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV262" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -39618,21 +40218,27 @@
       </c>
       <c r="BN264" t="inlineStr"/>
       <c r="BO264" t="n">
-        <v>0</v>
+        <v>8731610</v>
       </c>
       <c r="BP264" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ264" t="inlineStr"/>
+        <v>150430</v>
+      </c>
+      <c r="BQ264" t="n">
+        <v>58.04</v>
+      </c>
       <c r="BR264" t="inlineStr"/>
       <c r="BS264" t="inlineStr"/>
       <c r="BT264" t="n">
         <v>0</v>
       </c>
-      <c r="BU264" t="inlineStr"/>
+      <c r="BU264" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV264" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -39886,21 +40492,27 @@
       </c>
       <c r="BN266" t="inlineStr"/>
       <c r="BO266" t="n">
-        <v>0</v>
+        <v>7303830</v>
       </c>
       <c r="BP266" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ266" t="inlineStr"/>
+        <v>37100</v>
+      </c>
+      <c r="BQ266" t="n">
+        <v>196.87</v>
+      </c>
       <c r="BR266" t="inlineStr"/>
       <c r="BS266" t="inlineStr"/>
       <c r="BT266" t="n">
         <v>0</v>
       </c>
-      <c r="BU266" t="inlineStr"/>
+      <c r="BU266" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV266" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -40028,7 +40640,7 @@
       </c>
       <c r="BN267" t="inlineStr"/>
       <c r="BO267" t="n">
-        <v>0</v>
+        <v>1499630</v>
       </c>
       <c r="BP267" t="n">
         <v>0</v>
@@ -40039,10 +40651,14 @@
       <c r="BT267" t="n">
         <v>0</v>
       </c>
-      <c r="BU267" t="inlineStr"/>
+      <c r="BU267" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV267" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -40170,7 +40786,7 @@
       </c>
       <c r="BN268" t="inlineStr"/>
       <c r="BO268" t="n">
-        <v>0</v>
+        <v>1562480</v>
       </c>
       <c r="BP268" t="n">
         <v>0</v>
@@ -40181,10 +40797,14 @@
       <c r="BT268" t="n">
         <v>0</v>
       </c>
-      <c r="BU268" t="inlineStr"/>
+      <c r="BU268" t="inlineStr">
+        <is>
+          <t>元富</t>
+        </is>
+      </c>
       <c r="BV268" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -40564,7 +41184,7 @@
       </c>
       <c r="BN271" t="inlineStr"/>
       <c r="BO271" t="n">
-        <v>0</v>
+        <v>2548350</v>
       </c>
       <c r="BP271" t="n">
         <v>0</v>
@@ -40575,10 +41195,14 @@
       <c r="BT271" t="n">
         <v>0</v>
       </c>
-      <c r="BU271" t="inlineStr"/>
+      <c r="BU271" t="inlineStr">
+        <is>
+          <t>國泰</t>
+        </is>
+      </c>
       <c r="BV271" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -40968,21 +41592,27 @@
       </c>
       <c r="BN274" t="inlineStr"/>
       <c r="BO274" t="n">
-        <v>0</v>
+        <v>9478170</v>
       </c>
       <c r="BP274" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ274" t="inlineStr"/>
+        <v>20140</v>
+      </c>
+      <c r="BQ274" t="n">
+        <v>470.61</v>
+      </c>
       <c r="BR274" t="inlineStr"/>
       <c r="BS274" t="inlineStr"/>
       <c r="BT274" t="n">
         <v>0</v>
       </c>
-      <c r="BU274" t="inlineStr"/>
+      <c r="BU274" t="inlineStr">
+        <is>
+          <t>統一</t>
+        </is>
+      </c>
       <c r="BV274" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -41120,7 +41750,7 @@
       </c>
       <c r="BN275" t="inlineStr"/>
       <c r="BO275" t="n">
-        <v>0</v>
+        <v>6944990</v>
       </c>
       <c r="BP275" t="n">
         <v>0</v>
@@ -41131,10 +41761,14 @@
       <c r="BT275" t="n">
         <v>0</v>
       </c>
-      <c r="BU275" t="inlineStr"/>
+      <c r="BU275" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV275" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -41272,7 +41906,7 @@
       </c>
       <c r="BN276" t="inlineStr"/>
       <c r="BO276" t="n">
-        <v>0</v>
+        <v>822090</v>
       </c>
       <c r="BP276" t="n">
         <v>0</v>
@@ -41283,10 +41917,14 @@
       <c r="BT276" t="n">
         <v>0</v>
       </c>
-      <c r="BU276" t="inlineStr"/>
+      <c r="BU276" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV276" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -41424,7 +42062,7 @@
       </c>
       <c r="BN277" t="inlineStr"/>
       <c r="BO277" t="n">
-        <v>0</v>
+        <v>12822110</v>
       </c>
       <c r="BP277" t="n">
         <v>0</v>
@@ -41437,12 +42075,12 @@
       </c>
       <c r="BU277" t="inlineStr">
         <is>
-          <t>中信</t>
+          <t>富邦</t>
         </is>
       </c>
       <c r="BV277" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -41716,7 +42354,7 @@
       </c>
       <c r="BN279" t="inlineStr"/>
       <c r="BO279" t="n">
-        <v>0</v>
+        <v>99810</v>
       </c>
       <c r="BP279" t="n">
         <v>0</v>
@@ -41727,10 +42365,14 @@
       <c r="BT279" t="n">
         <v>0</v>
       </c>
-      <c r="BU279" t="inlineStr"/>
+      <c r="BU279" t="inlineStr">
+        <is>
+          <t>凱基</t>
+        </is>
+      </c>
       <c r="BV279" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -42004,21 +42646,27 @@
       </c>
       <c r="BN281" t="inlineStr"/>
       <c r="BO281" t="n">
-        <v>0</v>
+        <v>17931910</v>
       </c>
       <c r="BP281" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ281" t="inlineStr"/>
+        <v>162130</v>
+      </c>
+      <c r="BQ281" t="n">
+        <v>110.6</v>
+      </c>
       <c r="BR281" t="inlineStr"/>
       <c r="BS281" t="inlineStr"/>
       <c r="BT281" t="n">
         <v>0</v>
       </c>
-      <c r="BU281" t="inlineStr"/>
+      <c r="BU281" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV281" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -42272,21 +42920,27 @@
       </c>
       <c r="BN283" t="inlineStr"/>
       <c r="BO283" t="n">
-        <v>0</v>
+        <v>695420</v>
       </c>
       <c r="BP283" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ283" t="inlineStr"/>
+        <v>40600</v>
+      </c>
+      <c r="BQ283" t="n">
+        <v>17.13</v>
+      </c>
       <c r="BR283" t="inlineStr"/>
       <c r="BS283" t="inlineStr"/>
       <c r="BT283" t="n">
         <v>0</v>
       </c>
-      <c r="BU283" t="inlineStr"/>
+      <c r="BU283" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV283" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -42414,21 +43068,27 @@
       </c>
       <c r="BN284" t="inlineStr"/>
       <c r="BO284" t="n">
-        <v>0</v>
+        <v>6259170</v>
       </c>
       <c r="BP284" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ284" t="inlineStr"/>
+        <v>145780</v>
+      </c>
+      <c r="BQ284" t="n">
+        <v>42.94</v>
+      </c>
       <c r="BR284" t="inlineStr"/>
       <c r="BS284" t="inlineStr"/>
       <c r="BT284" t="n">
         <v>0</v>
       </c>
-      <c r="BU284" t="inlineStr"/>
+      <c r="BU284" t="inlineStr">
+        <is>
+          <t>兆豐</t>
+        </is>
+      </c>
       <c r="BV284" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -42556,7 +43216,7 @@
       </c>
       <c r="BN285" t="inlineStr"/>
       <c r="BO285" t="n">
-        <v>0</v>
+        <v>74370</v>
       </c>
       <c r="BP285" t="n">
         <v>0</v>
@@ -42567,10 +43227,14 @@
       <c r="BT285" t="n">
         <v>0</v>
       </c>
-      <c r="BU285" t="inlineStr"/>
+      <c r="BU285" t="inlineStr">
+        <is>
+          <t>永豐</t>
+        </is>
+      </c>
       <c r="BV285" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -42698,21 +43362,27 @@
       </c>
       <c r="BN286" t="inlineStr"/>
       <c r="BO286" t="n">
-        <v>0</v>
+        <v>16720700</v>
       </c>
       <c r="BP286" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ286" t="inlineStr"/>
+        <v>106230</v>
+      </c>
+      <c r="BQ286" t="n">
+        <v>157.4</v>
+      </c>
       <c r="BR286" t="inlineStr"/>
       <c r="BS286" t="inlineStr"/>
       <c r="BT286" t="n">
         <v>0</v>
       </c>
-      <c r="BU286" t="inlineStr"/>
+      <c r="BU286" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV286" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -43344,21 +44014,27 @@
       </c>
       <c r="BN291" t="inlineStr"/>
       <c r="BO291" t="n">
-        <v>0</v>
+        <v>14703320</v>
       </c>
       <c r="BP291" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ291" t="inlineStr"/>
+        <v>9800</v>
+      </c>
+      <c r="BQ291" t="n">
+        <v>1500.34</v>
+      </c>
       <c r="BR291" t="inlineStr"/>
       <c r="BS291" t="inlineStr"/>
       <c r="BT291" t="n">
         <v>0</v>
       </c>
-      <c r="BU291" t="inlineStr"/>
+      <c r="BU291" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV291" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -43486,7 +44162,7 @@
       </c>
       <c r="BN292" t="inlineStr"/>
       <c r="BO292" t="n">
-        <v>0</v>
+        <v>1619890</v>
       </c>
       <c r="BP292" t="n">
         <v>0</v>
@@ -43497,10 +44173,14 @@
       <c r="BT292" t="n">
         <v>0</v>
       </c>
-      <c r="BU292" t="inlineStr"/>
+      <c r="BU292" t="inlineStr">
+        <is>
+          <t>台新</t>
+        </is>
+      </c>
       <c r="BV292" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -43754,7 +44434,7 @@
       </c>
       <c r="BN294" t="inlineStr"/>
       <c r="BO294" t="n">
-        <v>0</v>
+        <v>867210</v>
       </c>
       <c r="BP294" t="n">
         <v>0</v>
@@ -43765,10 +44445,14 @@
       <c r="BT294" t="n">
         <v>0</v>
       </c>
-      <c r="BU294" t="inlineStr"/>
+      <c r="BU294" t="inlineStr">
+        <is>
+          <t>永豐</t>
+        </is>
+      </c>
       <c r="BV294" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -43896,21 +44580,27 @@
       </c>
       <c r="BN295" t="inlineStr"/>
       <c r="BO295" t="n">
-        <v>0</v>
+        <v>1458330</v>
       </c>
       <c r="BP295" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ295" t="inlineStr"/>
+        <v>140080</v>
+      </c>
+      <c r="BQ295" t="n">
+        <v>10.41</v>
+      </c>
       <c r="BR295" t="inlineStr"/>
       <c r="BS295" t="inlineStr"/>
       <c r="BT295" t="n">
         <v>0</v>
       </c>
-      <c r="BU295" t="inlineStr"/>
+      <c r="BU295" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV295" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -44038,7 +44728,7 @@
       </c>
       <c r="BN296" t="inlineStr"/>
       <c r="BO296" t="n">
-        <v>0</v>
+        <v>581090</v>
       </c>
       <c r="BP296" t="n">
         <v>0</v>
@@ -44049,10 +44739,14 @@
       <c r="BT296" t="n">
         <v>0</v>
       </c>
-      <c r="BU296" t="inlineStr"/>
+      <c r="BU296" t="inlineStr">
+        <is>
+          <t>元富</t>
+        </is>
+      </c>
       <c r="BV296" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -44306,7 +45000,7 @@
       </c>
       <c r="BN298" t="inlineStr"/>
       <c r="BO298" t="n">
-        <v>0</v>
+        <v>159520</v>
       </c>
       <c r="BP298" t="n">
         <v>0</v>
@@ -44317,10 +45011,14 @@
       <c r="BT298" t="n">
         <v>0</v>
       </c>
-      <c r="BU298" t="inlineStr"/>
+      <c r="BU298" t="inlineStr">
+        <is>
+          <t>國票</t>
+        </is>
+      </c>
       <c r="BV298" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -44448,7 +45146,7 @@
       </c>
       <c r="BN299" t="inlineStr"/>
       <c r="BO299" t="n">
-        <v>0</v>
+        <v>210620</v>
       </c>
       <c r="BP299" t="n">
         <v>0</v>
@@ -44459,10 +45157,14 @@
       <c r="BT299" t="n">
         <v>0</v>
       </c>
-      <c r="BU299" t="inlineStr"/>
+      <c r="BU299" t="inlineStr">
+        <is>
+          <t>統一</t>
+        </is>
+      </c>
       <c r="BV299" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -44842,7 +45544,7 @@
       </c>
       <c r="BN302" t="inlineStr"/>
       <c r="BO302" t="n">
-        <v>0</v>
+        <v>3808110</v>
       </c>
       <c r="BP302" t="n">
         <v>0</v>
@@ -44853,10 +45555,14 @@
       <c r="BT302" t="n">
         <v>0</v>
       </c>
-      <c r="BU302" t="inlineStr"/>
+      <c r="BU302" t="inlineStr">
+        <is>
+          <t>台新</t>
+        </is>
+      </c>
       <c r="BV302" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -44984,21 +45690,27 @@
       </c>
       <c r="BN303" t="inlineStr"/>
       <c r="BO303" t="n">
-        <v>0</v>
+        <v>1784860</v>
       </c>
       <c r="BP303" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ303" t="inlineStr"/>
+        <v>50050</v>
+      </c>
+      <c r="BQ303" t="n">
+        <v>35.66</v>
+      </c>
       <c r="BR303" t="inlineStr"/>
       <c r="BS303" t="inlineStr"/>
       <c r="BT303" t="n">
         <v>0</v>
       </c>
-      <c r="BU303" t="inlineStr"/>
+      <c r="BU303" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV303" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -45126,21 +45838,27 @@
       </c>
       <c r="BN304" t="inlineStr"/>
       <c r="BO304" t="n">
-        <v>0</v>
+        <v>1323200</v>
       </c>
       <c r="BP304" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ304" t="inlineStr"/>
+        <v>141070</v>
+      </c>
+      <c r="BQ304" t="n">
+        <v>9.380000000000001</v>
+      </c>
       <c r="BR304" t="inlineStr"/>
       <c r="BS304" t="inlineStr"/>
       <c r="BT304" t="n">
         <v>0</v>
       </c>
-      <c r="BU304" t="inlineStr"/>
+      <c r="BU304" t="inlineStr">
+        <is>
+          <t>統一</t>
+        </is>
+      </c>
       <c r="BV304" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -45646,7 +46364,7 @@
       </c>
       <c r="BN308" t="inlineStr"/>
       <c r="BO308" t="n">
-        <v>0</v>
+        <v>13110</v>
       </c>
       <c r="BP308" t="n">
         <v>0</v>
@@ -45657,10 +46375,14 @@
       <c r="BT308" t="n">
         <v>0</v>
       </c>
-      <c r="BU308" t="inlineStr"/>
+      <c r="BU308" t="inlineStr">
+        <is>
+          <t>元富</t>
+        </is>
+      </c>
       <c r="BV308" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -45788,21 +46510,27 @@
       </c>
       <c r="BN309" t="inlineStr"/>
       <c r="BO309" t="n">
-        <v>0</v>
+        <v>24351970</v>
       </c>
       <c r="BP309" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ309" t="inlineStr"/>
+        <v>798830</v>
+      </c>
+      <c r="BQ309" t="n">
+        <v>30.48</v>
+      </c>
       <c r="BR309" t="inlineStr"/>
       <c r="BS309" t="inlineStr"/>
       <c r="BT309" t="n">
         <v>0</v>
       </c>
-      <c r="BU309" t="inlineStr"/>
+      <c r="BU309" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV309" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -45930,7 +46658,7 @@
       </c>
       <c r="BN310" t="inlineStr"/>
       <c r="BO310" t="n">
-        <v>0</v>
+        <v>151230</v>
       </c>
       <c r="BP310" t="n">
         <v>0</v>
@@ -45941,10 +46669,14 @@
       <c r="BT310" t="n">
         <v>0</v>
       </c>
-      <c r="BU310" t="inlineStr"/>
+      <c r="BU310" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV310" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>
@@ -46072,7 +46804,7 @@
       </c>
       <c r="BN311" t="inlineStr"/>
       <c r="BO311" t="n">
-        <v>0</v>
+        <v>1336480</v>
       </c>
       <c r="BP311" t="n">
         <v>0</v>
@@ -46083,10 +46815,14 @@
       <c r="BT311" t="n">
         <v>0</v>
       </c>
-      <c r="BU311" t="inlineStr"/>
+      <c r="BU311" t="inlineStr">
+        <is>
+          <t>元大</t>
+        </is>
+      </c>
       <c r="BV311" t="inlineStr">
         <is>
-          <t>今日無可用權證成交金額</t>
+          <t>無明顯權證資金訊號</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update full daily pipeline with report artifacts
</commit_message>
<xml_diff>
--- a/output/latest/all_candidates_latest.xlsx
+++ b/output/latest/all_candidates_latest.xlsx
@@ -32382,17 +32382,17 @@
       </c>
       <c r="BN200" t="inlineStr"/>
       <c r="BO200" t="n">
-        <v>3520410</v>
+        <v>2992510</v>
       </c>
       <c r="BP200" t="n">
         <v>0</v>
       </c>
       <c r="BQ200" t="inlineStr"/>
       <c r="BR200" t="n">
-        <v>15.65</v>
+        <v>-1.69</v>
       </c>
       <c r="BS200" t="n">
-        <v>15.65</v>
+        <v>-1.69</v>
       </c>
       <c r="BT200" t="n">
         <v>0</v>
@@ -32532,17 +32532,17 @@
       </c>
       <c r="BN201" t="inlineStr"/>
       <c r="BO201" t="n">
-        <v>3045640</v>
+        <v>2705640</v>
       </c>
       <c r="BP201" t="n">
         <v>0</v>
       </c>
       <c r="BQ201" t="inlineStr"/>
       <c r="BR201" t="n">
-        <v>-49.04</v>
+        <v>-54.73</v>
       </c>
       <c r="BS201" t="n">
-        <v>-49.04</v>
+        <v>-54.73</v>
       </c>
       <c r="BT201" t="n">
         <v>0</v>
@@ -40034,37 +40034,17 @@
       <c r="BI255" t="inlineStr"/>
       <c r="BJ255" t="inlineStr"/>
       <c r="BK255" t="inlineStr"/>
-      <c r="BL255" t="inlineStr">
-        <is>
-          <t>no_signal</t>
-        </is>
-      </c>
-      <c r="BM255" t="n">
-        <v>0</v>
-      </c>
+      <c r="BL255" t="inlineStr"/>
+      <c r="BM255" t="inlineStr"/>
       <c r="BN255" t="inlineStr"/>
-      <c r="BO255" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP255" t="n">
-        <v>0</v>
-      </c>
+      <c r="BO255" t="inlineStr"/>
+      <c r="BP255" t="inlineStr"/>
       <c r="BQ255" t="inlineStr"/>
       <c r="BR255" t="inlineStr"/>
       <c r="BS255" t="inlineStr"/>
-      <c r="BT255" t="n">
-        <v>0</v>
-      </c>
-      <c r="BU255" t="inlineStr">
-        <is>
-          <t>元展</t>
-        </is>
-      </c>
-      <c r="BV255" t="inlineStr">
-        <is>
-          <t>今日無可用權證成交金額</t>
-        </is>
-      </c>
+      <c r="BT255" t="inlineStr"/>
+      <c r="BU255" t="inlineStr"/>
+      <c r="BV255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -50930,17 +50910,17 @@
       </c>
       <c r="BN333" t="inlineStr"/>
       <c r="BO333" t="n">
-        <v>3520410</v>
+        <v>2992510</v>
       </c>
       <c r="BP333" t="n">
         <v>0</v>
       </c>
       <c r="BQ333" t="inlineStr"/>
       <c r="BR333" t="n">
-        <v>15.65</v>
+        <v>-1.69</v>
       </c>
       <c r="BS333" t="n">
-        <v>15.65</v>
+        <v>-1.69</v>
       </c>
       <c r="BT333" t="n">
         <v>0</v>
@@ -56711,13 +56691,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="n">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>